<commit_message>
Tests actualizados: usercamerero usermaitre
</commit_message>
<xml_diff>
--- a/App/TestCases_App/User_camarero.xlsx
+++ b/App/TestCases_App/User_camarero.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\App\TestCases_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FCD955-06A5-45E4-8D79-88C084FAB7E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED49B579-44EE-4AE2-89C8-F0DF31AB3BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
   <si>
     <t>Num</t>
   </si>
@@ -199,7 +199,85 @@
     <t>No se puede buscar por fechas</t>
   </si>
   <si>
-    <t>Se ha introducido un númoro desorbitado de comensales, y al ir a pagar, se ha cerrado la aplicación.</t>
+    <t>Se ha introducido un número desorbitado de comensales, y al ir a pagar, se ha cerrado la aplicación.</t>
+  </si>
+  <si>
+    <t>BL</t>
+  </si>
+  <si>
+    <t>Take order: Add product</t>
+  </si>
+  <si>
+    <t>Take order: Delete product</t>
+  </si>
+  <si>
+    <t>The product is deleted</t>
+  </si>
+  <si>
+    <t>1. Select numbers of people
+2. Select products
+3. Clicks "+"
+4. Clicks "Añadir al pedido"</t>
+  </si>
+  <si>
+    <t>The product is added</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es necesario pulsar varias veces "Añadir al pedido" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select numbers of people
+2. Select products
+3. Clicks "-"
+</t>
+  </si>
+  <si>
+    <t>Take order: Cancel,add product</t>
+  </si>
+  <si>
+    <t>1. Select numbers of people
+2. Select products
+3. Clicks "+"
+4. Clicks "cancelar"</t>
+  </si>
+  <si>
+    <t>The operation is cancelled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es necesario pulsar varias veces "Cancelar" </t>
+  </si>
+  <si>
+    <t>Take order: print the order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select numbers of people
+2. Select products
+3. Clicks "Enviar comanda"
+</t>
+  </si>
+  <si>
+    <t>The order is sent</t>
+  </si>
+  <si>
+    <t>Tiene que poderse enviar a algun sitio: pdf, máquina, simulador..</t>
+  </si>
+  <si>
+    <t>USERCAM010</t>
+  </si>
+  <si>
+    <t>Change user</t>
+  </si>
+  <si>
+    <t>1. The user clicks "Cambiar de usuario"</t>
+  </si>
+  <si>
+    <t>1. The operation is done</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>USERCAM016</t>
   </si>
 </sst>
 </file>
@@ -302,7 +380,38 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6565"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -637,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -705,17 +814,21 @@
         <v>11</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+        <v>69</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>51</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
@@ -725,7 +838,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -734,10 +847,10 @@
         <v>23</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -745,21 +858,19 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>25</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="6" t="s">
         <v>23</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -767,10 +878,10 @@
         <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -778,7 +889,7 @@
         <v>23</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -789,10 +900,10 @@
         <v>15</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -800,7 +911,7 @@
         <v>23</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -811,17 +922,19 @@
         <v>16</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -831,15 +944,15 @@
         <v>17</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H9" s="7"/>
     </row>
@@ -851,10 +964,10 @@
         <v>18</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -865,16 +978,16 @@
     </row>
     <row r="11" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -891,90 +1004,164 @@
         <v>32</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="3"/>
+      <c r="C13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+      <c r="C14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="F14" s="3"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="6"/>
+      <c r="C15" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="H15" s="7"/>
     </row>
-    <row r="16" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="F16" s="3"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="7"/>
+      <c r="G16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G16">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PTE">
+  <conditionalFormatting sqref="G2 G4:G17">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="PTE">
       <formula>NOT(ISERROR(SEARCH("PTE",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="BL">
+    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="BL">
       <formula>NOT(ISERROR(SEARCH("BL",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="KO">
+    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="KO">
       <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
     </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="OK">
+      <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PTE">
+      <formula>NOT(ISERROR(SEARCH("PTE",G3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="BL">
+      <formula>NOT(ISERROR(SEARCH("BL",G3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="KO">
+      <formula>NOT(ISERROR(SEARCH("KO",G3)))</formula>
+    </cfRule>
     <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="OK">
-      <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("OK",G3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>